<commit_message>
Update inventory workbook display and reload behavior
</commit_message>
<xml_diff>
--- a/2602_inventory.xlsx
+++ b/2602_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cursor_work_space\Working Capital Dashboard\cashflow\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{719B9AF0-10EB-4906-9283-238FADCE2F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1998E3FA-7AD4-46D4-9135-1AE32D5E1FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="26430" windowHeight="16440" xr2:uid="{D593AF19-A322-4513-BC5A-A55E0694C254}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t>구분</t>
   </si>
@@ -112,6 +112,12 @@
   <si>
     <t>재고주수</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>판매율</t>
+  </si>
+  <si>
+    <t>재고주수</t>
   </si>
 </sst>
 </file>
@@ -645,7 +651,7 @@
     <col min="11" max="11" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="33.75" thickBot="1">
+    <row r="1" spans="1:15" ht="17.25" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -707,7 +713,7 @@
         <v>214752.25308737866</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H2" s="5">
         <v>214752.25308737866</v>
@@ -725,10 +731,10 @@
         <v>96010.846325011575</v>
       </c>
       <c r="M2" s="5">
-        <v>127385.34165361986</v>
+        <v>141477.51871815659</v>
       </c>
       <c r="N2" s="5">
-        <v>185140.60567139171</v>
+        <v>171048.42860685498</v>
       </c>
       <c r="O2" s="7" t="s">
         <v>22</v>
@@ -776,6 +782,7 @@
         <v>32184.425330851984</v>
       </c>
       <c r="O3" s="7">
+        <f t="shared" ref="O3:O8" si="0">+(J3+M3)/(H3+I3+L3)</f>
         <v>0.56083613388131059</v>
       </c>
     </row>
@@ -817,13 +824,14 @@
         <v>11011.818452380954</v>
       </c>
       <c r="M4" s="10">
-        <v>30474.853982909903</v>
+        <v>42567.031047446617</v>
       </c>
       <c r="N4" s="10">
-        <v>21704.277469471053</v>
+        <v>9612.1004049343392</v>
       </c>
       <c r="O4" s="7">
-        <v>0.65453384923505353</v>
+        <f t="shared" si="0"/>
+        <v>0.84700456707993899</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="17.25" thickBot="1">
@@ -858,13 +866,14 @@
       </c>
       <c r="L5" s="9"/>
       <c r="M5" s="10">
-        <v>30311.959247120481</v>
+        <v>32311.959247120481</v>
       </c>
       <c r="N5" s="10">
-        <v>25994.254752879511</v>
+        <v>23994.254752879511</v>
       </c>
       <c r="O5" s="7">
-        <v>0.64408585128480333</v>
+        <f t="shared" si="0"/>
+        <v>0.67200340115585488</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="17.25" thickBot="1">
@@ -905,6 +914,7 @@
         <v>44642.332835611393</v>
       </c>
       <c r="O6" s="7">
+        <f t="shared" si="0"/>
         <v>0.33949105227762322</v>
       </c>
     </row>
@@ -948,6 +958,7 @@
         <v>11093.355569252424</v>
       </c>
       <c r="O7" s="7">
+        <f t="shared" si="0"/>
         <v>5.2929899680132883E-2</v>
       </c>
     </row>
@@ -989,6 +1000,7 @@
         <v>49521.959713325326</v>
       </c>
       <c r="O8" s="7">
+        <f t="shared" si="0"/>
         <v>0.24568525779359018</v>
       </c>
     </row>
@@ -1012,7 +1024,7 @@
         <v>148512.38437864077</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H9" s="5">
         <v>148512.38437864077</v>
@@ -1030,10 +1042,10 @@
         <v>168731.57696526911</v>
       </c>
       <c r="M9" s="5">
-        <v>150913.12570997101</v>
+        <v>136821.12570997101</v>
       </c>
       <c r="N9" s="5">
-        <v>154256.84725529805</v>
+        <v>168348.84725529805</v>
       </c>
       <c r="O9" s="12" t="s">
         <v>23</v>
@@ -1077,13 +1089,14 @@
         <v>74197.777279589573</v>
       </c>
       <c r="M10" s="10">
-        <v>68666.636385592792</v>
+        <v>63666.636385592792</v>
       </c>
       <c r="N10" s="10">
-        <v>61723.881893996775</v>
+        <v>66723.881893996775</v>
       </c>
       <c r="O10" s="12">
-        <v>37.004943638780091</v>
+        <f>+N10/(M10+J10)*52</f>
+        <v>42.449637578796874</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="17.25" thickBot="1">
@@ -1124,13 +1137,14 @@
         <v>74413.471821727158</v>
       </c>
       <c r="M11" s="10">
-        <v>59157.792212302724</v>
+        <v>57065.792212302724</v>
       </c>
       <c r="N11" s="10">
-        <v>73497.483609424424</v>
+        <v>75589.483609424424</v>
       </c>
       <c r="O11" s="12">
-        <v>51.000587990866201</v>
+        <f>+N11/(M11+J11)*52</f>
+        <v>53.958581280084346</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="17.25" thickBot="1">
@@ -1171,13 +1185,14 @@
         <v>17557.526911571415</v>
       </c>
       <c r="M12" s="10">
-        <v>21178.157019052589</v>
+        <v>14178.157019052589</v>
       </c>
       <c r="N12" s="10">
-        <v>15023.130892518828</v>
+        <v>22023.130892518828</v>
       </c>
       <c r="O12" s="12">
-        <v>31.197408743934133</v>
+        <f>+N12/(M12+J12)*52</f>
+        <v>63.479087533584227</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="17.25" thickBot="1">
@@ -1224,6 +1239,7 @@
         <v>4012.350859358045</v>
       </c>
       <c r="O13" s="12">
+        <f>+N13/(M13+J13)*52</f>
         <v>43.011843754930453</v>
       </c>
     </row>
@@ -1263,10 +1279,10 @@
         <v>264742.42329028068</v>
       </c>
       <c r="M14" s="5">
-        <v>278298.46736359084</v>
+        <v>278298.64442812756</v>
       </c>
       <c r="N14" s="5">
-        <v>339397.45292668976</v>
+        <v>339397.27586215304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update inventory workbook data
</commit_message>
<xml_diff>
--- a/2602_inventory.xlsx
+++ b/2602_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cursor_work_space\Working Capital Dashboard\cashflow\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48427C41-EC9D-4350-AC2D-B5184814ED5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC4727C-153D-4A2E-84FD-542AD823EE4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="26430" windowHeight="16440" xr2:uid="{D593AF19-A322-4513-BC5A-A55E0694C254}"/>
   </bookViews>
@@ -98,14 +98,6 @@
     <t>Total</t>
   </si>
   <si>
-    <t>판매가능</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>26년 2월말</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>판매율</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -118,6 +110,12 @@
   </si>
   <si>
     <t>재고주수</t>
+  </si>
+  <si>
+    <t>판매가능</t>
+  </si>
+  <si>
+    <t>26년 2월말</t>
   </si>
 </sst>
 </file>
@@ -662,7 +660,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
@@ -681,7 +679,7 @@
         <v>3</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>2</v>
@@ -713,13 +711,13 @@
         <v>214752.25308737866</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H2" s="5">
-        <v>214752.25308737866</v>
+        <v>203512.30156310683</v>
       </c>
       <c r="I2" s="5">
-        <v>40574.291046728154</v>
+        <v>61814.242571000002</v>
       </c>
       <c r="J2" s="5">
         <v>40414.686814000001</v>
@@ -731,13 +729,13 @@
         <v>96010.846325011575</v>
       </c>
       <c r="M2" s="5">
-        <v>155477.51871815659</v>
+        <v>149896.33510990415</v>
       </c>
       <c r="N2" s="5">
-        <v>157048.42860685498</v>
+        <v>162629.61221510742</v>
       </c>
       <c r="O2" s="7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="17.25" thickBot="1">
@@ -808,11 +806,9 @@
       <c r="G4" s="11">
         <v>0.58201228178707043</v>
       </c>
-      <c r="H4" s="9">
-        <v>11239.951524271846</v>
-      </c>
+      <c r="H4" s="9"/>
       <c r="I4" s="9">
-        <v>40574.291046728154</v>
+        <v>61814.242571000002</v>
       </c>
       <c r="J4" s="9">
         <v>10646.929570999999</v>
@@ -824,14 +820,14 @@
         <v>11011.818452380954</v>
       </c>
       <c r="M4" s="10">
-        <v>42567.031047446617</v>
+        <v>44985.847439194178</v>
       </c>
       <c r="N4" s="10">
-        <v>9612.1004049343392</v>
+        <v>7193.2840131867779</v>
       </c>
       <c r="O4" s="7">
         <f t="shared" si="0"/>
-        <v>0.84700456707993899</v>
+        <v>0.76391303097298047</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="17.25" thickBot="1">
@@ -866,14 +862,14 @@
       </c>
       <c r="L5" s="9"/>
       <c r="M5" s="10">
-        <v>39311.959247120481</v>
+        <v>34311.959247120481</v>
       </c>
       <c r="N5" s="10">
-        <v>16994.254752879511</v>
+        <v>21994.254752879511</v>
       </c>
       <c r="O5" s="7">
         <f t="shared" si="0"/>
-        <v>0.7697148257045352</v>
+        <v>0.69992095102690632</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="17.25" thickBot="1">
@@ -908,14 +904,14 @@
       </c>
       <c r="L6" s="9"/>
       <c r="M6" s="10">
-        <v>22953.460164388609</v>
+        <v>19953.460164388609</v>
       </c>
       <c r="N6" s="10">
-        <v>37642.332835611393</v>
+        <v>40642.332835611393</v>
       </c>
       <c r="O6" s="7">
         <f t="shared" si="0"/>
-        <v>0.44183852467985868</v>
+        <v>0.39797532222175774</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="17.25" thickBot="1">
@@ -1024,7 +1020,7 @@
         <v>148512.38437864077</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H9" s="5">
         <v>148512.38437864077</v>
@@ -1039,16 +1035,16 @@
         <v>136438.39599999998</v>
       </c>
       <c r="L9" s="5">
-        <v>168731.57696526911</v>
+        <v>126612.37997057514</v>
       </c>
       <c r="M9" s="5">
-        <v>158013.12570997101</v>
+        <v>129013.12570997102</v>
       </c>
       <c r="N9" s="5">
-        <v>147156.84725529805</v>
+        <v>134037.6502606041</v>
       </c>
       <c r="O9" s="12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="17.25" thickBot="1">
@@ -1086,17 +1082,17 @@
         <v>56192.741000000002</v>
       </c>
       <c r="L10" s="9">
-        <v>74197.777279589573</v>
+        <v>56731.54785750981</v>
       </c>
       <c r="M10" s="10">
-        <v>68666.636385592792</v>
+        <v>45666.636385592792</v>
       </c>
       <c r="N10" s="10">
-        <v>61723.881893996775</v>
+        <v>67257.652471917027</v>
       </c>
       <c r="O10" s="12">
         <f>+N10/(M10+J10)*52</f>
-        <v>37.004943638780091</v>
+        <v>54.873635052788899</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="17.25" thickBot="1">
@@ -1134,17 +1130,17 @@
         <v>58241.803999999996</v>
       </c>
       <c r="L11" s="9">
-        <v>74413.471821727158</v>
+        <v>53878.318068063025</v>
       </c>
       <c r="M11" s="10">
-        <v>72157.792212302724</v>
+        <v>67157.792212302724</v>
       </c>
       <c r="N11" s="10">
-        <v>60497.483609424424</v>
+        <v>44962.329855760298</v>
       </c>
       <c r="O11" s="12">
         <f>+N11/(M11+J11)*52</f>
-        <v>35.773820269944629</v>
+        <v>28.190314346782486</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="17.25" thickBot="1">
@@ -1182,17 +1178,17 @@
         <v>18643.760999999999</v>
       </c>
       <c r="L12" s="9">
-        <v>17557.526911571415</v>
+        <v>13439.713092621341</v>
       </c>
       <c r="M12" s="10">
-        <v>15178.157019052589</v>
+        <v>14178.157019052589</v>
       </c>
       <c r="N12" s="10">
-        <v>21023.130892518828</v>
+        <v>17905.317073568753</v>
       </c>
       <c r="O12" s="12">
         <f>+N12/(M12+J12)*52</f>
-        <v>57.414210461652971</v>
+        <v>51.609972958738311</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="17.25" thickBot="1">
@@ -1264,10 +1260,10 @@
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="5">
-        <v>363264.63746601943</v>
+        <v>352024.68594174762</v>
       </c>
       <c r="I14" s="5">
-        <v>69151.852415087371</v>
+        <v>90391.803939359219</v>
       </c>
       <c r="J14" s="5">
         <v>81066.236560999998</v>
@@ -1276,13 +1272,13 @@
         <v>352953.49699999997</v>
       </c>
       <c r="L14" s="5">
-        <v>264742.42329028068</v>
+        <v>222623.22629558673</v>
       </c>
       <c r="M14" s="5">
-        <v>313490.64442812756</v>
+        <v>278909.46081987518</v>
       </c>
       <c r="N14" s="5">
-        <v>304205.27586215304</v>
+        <v>296667.26247571153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update inventory workbook and UI highlights
</commit_message>
<xml_diff>
--- a/2602_inventory.xlsx
+++ b/2602_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cursor_work_space\Working Capital Dashboard\cashflow\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CEAB571-A231-4111-AA96-E9E2E563A546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBAA4D41-E09C-40F7-A548-B07B0FE96772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="26430" windowHeight="16440" xr2:uid="{D593AF19-A322-4513-BC5A-A55E0694C254}"/>
   </bookViews>
@@ -259,34 +259,6 @@
   </si>
   <si>
     <r>
-      <t>당년</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF475569"/>
-        <rFont val="Segoe UI"/>
-        <family val="2"/>
-      </rPr>
-      <t>F</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>당년</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF475569"/>
-        <rFont val="Segoe UI"/>
-        <family val="2"/>
-      </rPr>
-      <t>S</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>1</t>
     </r>
     <r>
@@ -330,6 +302,12 @@
       </rPr>
       <t>합계</t>
     </r>
+  </si>
+  <si>
+    <t>당년F</t>
+  </si>
+  <si>
+    <t>당년S</t>
   </si>
 </sst>
 </file>
@@ -971,13 +949,13 @@
         <v>216515</v>
       </c>
       <c r="L2" s="5">
-        <v>106011</v>
+        <v>112011</v>
       </c>
       <c r="M2" s="5">
         <v>149896</v>
       </c>
       <c r="N2" s="5">
-        <v>172630</v>
+        <v>178630</v>
       </c>
       <c r="O2" s="7" t="s">
         <v>11</v>
@@ -985,7 +963,7 @@
     </row>
     <row r="3" spans="1:15" ht="17.25" thickBot="1">
       <c r="A3" s="17" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B3" s="9">
         <v>0</v>
@@ -1031,7 +1009,7 @@
     </row>
     <row r="4" spans="1:15" ht="17.25" thickBot="1">
       <c r="A4" s="17" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9">
@@ -1060,22 +1038,22 @@
         <v>41167</v>
       </c>
       <c r="L4" s="9">
-        <v>21012</v>
+        <v>27012</v>
       </c>
       <c r="M4" s="10">
         <v>44986</v>
       </c>
       <c r="N4" s="10">
-        <v>17193</v>
+        <v>23193</v>
       </c>
       <c r="O4" s="7">
         <f t="shared" si="0"/>
-        <v>0.76391673303490515</v>
+        <v>0.70576966990586865</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="17.25" thickBot="1">
       <c r="A5" s="8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" s="9">
         <v>116967</v>
@@ -1117,7 +1095,7 @@
     </row>
     <row r="6" spans="1:15" ht="17.25" thickBot="1">
       <c r="A6" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B6" s="9">
         <v>72725</v>
@@ -1245,7 +1223,7 @@
     </row>
     <row r="9" spans="1:15" ht="17.25" thickBot="1">
       <c r="A9" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="5">
         <v>168561</v>
@@ -1515,13 +1493,13 @@
         <v>352953</v>
       </c>
       <c r="L14" s="5">
-        <v>232623</v>
+        <v>238623</v>
       </c>
       <c r="M14" s="5">
         <v>278909</v>
       </c>
       <c r="N14" s="5">
-        <v>306667</v>
+        <v>312667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>